<commit_message>
Acero con marco unico en tramo normal y motos (doble solo en camiones), verificacion de velocidades y autolimpieza CE.040, marco normativo en memoria y Word
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/MEMORIA_CALCULO_COLECTOR_HOGAR_REFUGIO.xlsx
+++ b/entregables/MEMORIA_CALCULO_COLECTOR_HOGAR_REFUGIO.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -589,7 +589,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Losa superior e = 0.10 (tramo normal y cruce de motos) y e = 0.25 en el cruce de camiones; muros e = 0.15 (altura interior 1.40 a 1.65 m) como marco cerrado monolitico; losa de fondo e = 0.15; tapas de registro 0.68 x 0.68 x 0.08.</t>
+          <t>Marco cerrado monolitico: losa superior e = 0.10, muros e = 0.15 (altura interior 1.40 a 1.65 m) y losa de fondo e = 0.15 con un solo marco 3/8" @0.20 en el eje de la seccion y longitudinales 3/8" @0.25 (una capa; E.060 14.3.4); cruce de motos marco 3/8" @0.15; cruce de camiones losas e = 0.25 y doble marco 1/2" @0.15 (una capa en cada cara). Tapas de registro 0.68 x 0.68 x 0.08.</t>
         </is>
       </c>
     </row>
@@ -708,60 +708,71 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Cunetas con caida libre al colector (de 6)</t>
-        </is>
-      </c>
-      <c r="B20" s="10">
-        <f>COUNTIF(CUNETAS!L5:L10,"CAIDA LIBRE")</f>
+          <t>Velocidades y autolimpieza (0.90 a 3.0 m/s; tau &gt;= 0.15 kg/m2)</t>
+        </is>
+      </c>
+      <c r="B20" s="8">
+        <f>PERFIL_FLUJO!B200</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Resalto en la poza de la caja de caida</t>
-        </is>
-      </c>
-      <c r="B21" s="8">
-        <f>EMPALME!B19</f>
+          <t>Cunetas con caida libre al colector (de 6)</t>
+        </is>
+      </c>
+      <c r="B21" s="10">
+        <f>COUNTIF(CUNETAS!L5:L10,"CAIDA LIBRE")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>Resalto en la poza de la caja de caida</t>
+        </is>
+      </c>
+      <c r="B22" s="8">
+        <f>EMPALME!B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>Elementos estructurales que no cumplen</t>
         </is>
       </c>
-      <c r="B22" s="10">
+      <c r="B23" s="10">
         <f>COUNTIF(ESTRUCTURAL!E:E,"NO CUMPLE")</f>
         <v/>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>NOTAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>La cota de llegada del CAR Varones (260.18) es un supuesto (260.69 - 0.5 % x 102.36 m) y debe confirmarse con el proyecto CUI 2705619; solo afecta a la altura de la caida en la caja de llegada.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>La ubicacion UTM es referencial: el plano de arquitectura se georreferencio haciendo coincidir el R-01 del CAR Mujeres con la esquina sur-oeste del frente y el rumbo del lindero (azimut 49.54). Verificar en campo.</t>
+          <t>La cota de llegada del CAR Varones (260.18) es un supuesto (260.69 - 0.5 % x 102.36 m) y debe confirmarse con el proyecto CUI 2705619; solo afecta a la altura de la caida en la caja de llegada.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>La ubicacion UTM es referencial: el plano de arquitectura se georreferencio haciendo coincidir el R-01 del CAR Mujeres con la esquina sur-oeste del frente y el rumbo del lindero (azimut 49.54). Verificar en campo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Las cunetas de arquitectura se toman como dato (perfiles 01 a 12 del plano PLANTA GENERAL REFUGIO, version 03-10-2026).</t>
         </is>
@@ -28574,21 +28585,671 @@
       </c>
     </row>
     <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>VERIFICACION DE VELOCIDADES Y AUTOLIMPIEZA (RNE CE.040 Drenaje Pluvial; esfuerzo tractivo minimo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Tirante normal por punto fijo: y(k+1) = (Q n (b + 2 y(k))^(2/3) / (b^(5/3) S^(1/2)))^(3/5), 8 iteraciones (columnas P a W). Esfuerzo tractivo tau = gamma R S.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="11" t="inlineStr">
+        <is>
+          <t>CASO</t>
+        </is>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>Q (m3/s)</t>
+        </is>
+      </c>
+      <c r="C101" s="11" t="inlineStr">
+        <is>
+          <t>yn (m)</t>
+        </is>
+      </c>
+      <c r="D101" s="11" t="inlineStr">
+        <is>
+          <t>V (m/s)</t>
+        </is>
+      </c>
+      <c r="E101" s="11" t="inlineStr">
+        <is>
+          <t>R (m)</t>
+        </is>
+      </c>
+      <c r="F101" s="11" t="inlineStr">
+        <is>
+          <t>TAU (kg/m2)</t>
+        </is>
+      </c>
+      <c r="G101" s="11" t="inlineStr">
+        <is>
+          <t>TAU (Pa)</t>
+        </is>
+      </c>
+      <c r="H101" s="11" t="inlineStr">
+        <is>
+          <t>FROUDE</t>
+        </is>
+      </c>
+      <c r="I101" s="11" t="inlineStr">
+        <is>
+          <t>V &gt;= 0.90 m/s (CE.040)</t>
+        </is>
+      </c>
+      <c r="J101" s="11" t="inlineStr">
+        <is>
+          <t>TAU &gt;= 0.15 kg/m2</t>
+        </is>
+      </c>
+      <c r="K101" s="11" t="inlineStr">
+        <is>
+          <t>V &lt;= 3.0 m/s (concreto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>Caudal de diseno del tramo (Varones + Refugio)</t>
+        </is>
+      </c>
+      <c r="B102" s="24">
+        <f>CAUDALES!$B$13</f>
+        <v/>
+      </c>
+      <c r="C102" s="16">
+        <f>W102</f>
+        <v/>
+      </c>
+      <c r="D102" s="19">
+        <f>B102/(DATOS!$B$14*C102)</f>
+        <v/>
+      </c>
+      <c r="E102" s="16">
+        <f>DATOS!$B$14*C102/(DATOS!$B$14+2*C102)</f>
+        <v/>
+      </c>
+      <c r="F102" s="16">
+        <f>1000*E102*DATOS!$B$20</f>
+        <v/>
+      </c>
+      <c r="G102" s="19">
+        <f>F102*9.81</f>
+        <v/>
+      </c>
+      <c r="H102" s="19">
+        <f>D102/SQRT(9.81*C102)</f>
+        <v/>
+      </c>
+      <c r="I102" s="5">
+        <f>IF(D102&gt;=0.9,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="J102" s="5">
+        <f>IF(F102&gt;=0.15,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="K102" s="5">
+        <f>IF(D102&lt;=3.0,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="P102" s="20">
+        <f>(B102*DATOS!$B$31/(DATOS!$B$14*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="Q102" s="20">
+        <f>(B102*DATOS!$B$31*(DATOS!$B$14+2*P102)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="R102" s="20">
+        <f>(B102*DATOS!$B$31*(DATOS!$B$14+2*Q102)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="S102" s="20">
+        <f>(B102*DATOS!$B$31*(DATOS!$B$14+2*R102)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="T102" s="20">
+        <f>(B102*DATOS!$B$31*(DATOS!$B$14+2*S102)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="U102" s="20">
+        <f>(B102*DATOS!$B$31*(DATOS!$B$14+2*T102)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="V102" s="20">
+        <f>(B102*DATOS!$B$31*(DATOS!$B$14+2*U102)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="W102" s="20">
+        <f>(B102*DATOS!$B$31*(DATOS!$B$14+2*V102)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>Solo aporte de CAR Varones (CUI 2705619)</t>
+        </is>
+      </c>
+      <c r="B103" s="24">
+        <f>CAUDALES!$B$10/1000</f>
+        <v/>
+      </c>
+      <c r="C103" s="16">
+        <f>W103</f>
+        <v/>
+      </c>
+      <c r="D103" s="19">
+        <f>B103/(DATOS!$B$14*C103)</f>
+        <v/>
+      </c>
+      <c r="E103" s="16">
+        <f>DATOS!$B$14*C103/(DATOS!$B$14+2*C103)</f>
+        <v/>
+      </c>
+      <c r="F103" s="16">
+        <f>1000*E103*DATOS!$B$20</f>
+        <v/>
+      </c>
+      <c r="G103" s="19">
+        <f>F103*9.81</f>
+        <v/>
+      </c>
+      <c r="H103" s="19">
+        <f>D103/SQRT(9.81*C103)</f>
+        <v/>
+      </c>
+      <c r="I103" s="5">
+        <f>IF(D103&gt;=0.9,"CUMPLE","caudal parcial: ver tau")</f>
+        <v/>
+      </c>
+      <c r="J103" s="5">
+        <f>IF(F103&gt;=0.15,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="K103" s="5">
+        <f>IF(D103&lt;=3.0,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="P103" s="20">
+        <f>(B103*DATOS!$B$31/(DATOS!$B$14*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="Q103" s="20">
+        <f>(B103*DATOS!$B$31*(DATOS!$B$14+2*P103)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="R103" s="20">
+        <f>(B103*DATOS!$B$31*(DATOS!$B$14+2*Q103)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="S103" s="20">
+        <f>(B103*DATOS!$B$31*(DATOS!$B$14+2*R103)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="T103" s="20">
+        <f>(B103*DATOS!$B$31*(DATOS!$B$14+2*S103)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="U103" s="20">
+        <f>(B103*DATOS!$B$31*(DATOS!$B$14+2*T103)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="V103" s="20">
+        <f>(B103*DATOS!$B$31*(DATOS!$B$14+2*U103)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="W103" s="20">
+        <f>(B103*DATOS!$B$31*(DATOS!$B$14+2*V103)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>Solo aporte del Hogar de Refugio (CUI 2675514)</t>
+        </is>
+      </c>
+      <c r="B104" s="24">
+        <f>CAUDALES!$B$11/1000</f>
+        <v/>
+      </c>
+      <c r="C104" s="16">
+        <f>W104</f>
+        <v/>
+      </c>
+      <c r="D104" s="19">
+        <f>B104/(DATOS!$B$14*C104)</f>
+        <v/>
+      </c>
+      <c r="E104" s="16">
+        <f>DATOS!$B$14*C104/(DATOS!$B$14+2*C104)</f>
+        <v/>
+      </c>
+      <c r="F104" s="16">
+        <f>1000*E104*DATOS!$B$20</f>
+        <v/>
+      </c>
+      <c r="G104" s="19">
+        <f>F104*9.81</f>
+        <v/>
+      </c>
+      <c r="H104" s="19">
+        <f>D104/SQRT(9.81*C104)</f>
+        <v/>
+      </c>
+      <c r="I104" s="5">
+        <f>IF(D104&gt;=0.9,"CUMPLE","caudal parcial: ver tau")</f>
+        <v/>
+      </c>
+      <c r="J104" s="5">
+        <f>IF(F104&gt;=0.15,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="K104" s="5">
+        <f>IF(D104&lt;=3.0,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="P104" s="20">
+        <f>(B104*DATOS!$B$31/(DATOS!$B$14*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="Q104" s="20">
+        <f>(B104*DATOS!$B$31*(DATOS!$B$14+2*P104)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="R104" s="20">
+        <f>(B104*DATOS!$B$31*(DATOS!$B$14+2*Q104)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="S104" s="20">
+        <f>(B104*DATOS!$B$31*(DATOS!$B$14+2*R104)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="T104" s="20">
+        <f>(B104*DATOS!$B$31*(DATOS!$B$14+2*S104)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="U104" s="20">
+        <f>(B104*DATOS!$B$31*(DATOS!$B$14+2*T104)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="V104" s="20">
+        <f>(B104*DATOS!$B$31*(DATOS!$B$14+2*U104)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="W104" s="20">
+        <f>(B104*DATOS!$B$31*(DATOS!$B$14+2*V104)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>50 % del caudal de diseno</t>
+        </is>
+      </c>
+      <c r="B105" s="24">
+        <f>0.50*CAUDALES!$B$13</f>
+        <v/>
+      </c>
+      <c r="C105" s="16">
+        <f>W105</f>
+        <v/>
+      </c>
+      <c r="D105" s="19">
+        <f>B105/(DATOS!$B$14*C105)</f>
+        <v/>
+      </c>
+      <c r="E105" s="16">
+        <f>DATOS!$B$14*C105/(DATOS!$B$14+2*C105)</f>
+        <v/>
+      </c>
+      <c r="F105" s="16">
+        <f>1000*E105*DATOS!$B$20</f>
+        <v/>
+      </c>
+      <c r="G105" s="19">
+        <f>F105*9.81</f>
+        <v/>
+      </c>
+      <c r="H105" s="19">
+        <f>D105/SQRT(9.81*C105)</f>
+        <v/>
+      </c>
+      <c r="I105" s="5">
+        <f>IF(D105&gt;=0.9,"CUMPLE","caudal parcial: ver tau")</f>
+        <v/>
+      </c>
+      <c r="J105" s="5">
+        <f>IF(F105&gt;=0.15,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="K105" s="5">
+        <f>IF(D105&lt;=3.0,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="P105" s="20">
+        <f>(B105*DATOS!$B$31/(DATOS!$B$14*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="Q105" s="20">
+        <f>(B105*DATOS!$B$31*(DATOS!$B$14+2*P105)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="R105" s="20">
+        <f>(B105*DATOS!$B$31*(DATOS!$B$14+2*Q105)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="S105" s="20">
+        <f>(B105*DATOS!$B$31*(DATOS!$B$14+2*R105)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="T105" s="20">
+        <f>(B105*DATOS!$B$31*(DATOS!$B$14+2*S105)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="U105" s="20">
+        <f>(B105*DATOS!$B$31*(DATOS!$B$14+2*T105)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="V105" s="20">
+        <f>(B105*DATOS!$B$31*(DATOS!$B$14+2*U105)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="W105" s="20">
+        <f>(B105*DATOS!$B$31*(DATOS!$B$14+2*V105)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>25 % del caudal de diseno</t>
+        </is>
+      </c>
+      <c r="B106" s="24">
+        <f>0.25*CAUDALES!$B$13</f>
+        <v/>
+      </c>
+      <c r="C106" s="16">
+        <f>W106</f>
+        <v/>
+      </c>
+      <c r="D106" s="19">
+        <f>B106/(DATOS!$B$14*C106)</f>
+        <v/>
+      </c>
+      <c r="E106" s="16">
+        <f>DATOS!$B$14*C106/(DATOS!$B$14+2*C106)</f>
+        <v/>
+      </c>
+      <c r="F106" s="16">
+        <f>1000*E106*DATOS!$B$20</f>
+        <v/>
+      </c>
+      <c r="G106" s="19">
+        <f>F106*9.81</f>
+        <v/>
+      </c>
+      <c r="H106" s="19">
+        <f>D106/SQRT(9.81*C106)</f>
+        <v/>
+      </c>
+      <c r="I106" s="5">
+        <f>IF(D106&gt;=0.9,"CUMPLE","caudal parcial: ver tau")</f>
+        <v/>
+      </c>
+      <c r="J106" s="5">
+        <f>IF(F106&gt;=0.15,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="K106" s="5">
+        <f>IF(D106&lt;=3.0,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="P106" s="20">
+        <f>(B106*DATOS!$B$31/(DATOS!$B$14*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="Q106" s="20">
+        <f>(B106*DATOS!$B$31*(DATOS!$B$14+2*P106)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="R106" s="20">
+        <f>(B106*DATOS!$B$31*(DATOS!$B$14+2*Q106)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="S106" s="20">
+        <f>(B106*DATOS!$B$31*(DATOS!$B$14+2*R106)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="T106" s="20">
+        <f>(B106*DATOS!$B$31*(DATOS!$B$14+2*S106)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="U106" s="20">
+        <f>(B106*DATOS!$B$31*(DATOS!$B$14+2*T106)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="V106" s="20">
+        <f>(B106*DATOS!$B$31*(DATOS!$B$14+2*U106)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="W106" s="20">
+        <f>(B106*DATOS!$B$31*(DATOS!$B$14+2*V106)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>10 % del caudal de diseno (lluvia menor)</t>
+        </is>
+      </c>
+      <c r="B107" s="24">
+        <f>0.10*CAUDALES!$B$13</f>
+        <v/>
+      </c>
+      <c r="C107" s="16">
+        <f>W107</f>
+        <v/>
+      </c>
+      <c r="D107" s="19">
+        <f>B107/(DATOS!$B$14*C107)</f>
+        <v/>
+      </c>
+      <c r="E107" s="16">
+        <f>DATOS!$B$14*C107/(DATOS!$B$14+2*C107)</f>
+        <v/>
+      </c>
+      <c r="F107" s="16">
+        <f>1000*E107*DATOS!$B$20</f>
+        <v/>
+      </c>
+      <c r="G107" s="19">
+        <f>F107*9.81</f>
+        <v/>
+      </c>
+      <c r="H107" s="19">
+        <f>D107/SQRT(9.81*C107)</f>
+        <v/>
+      </c>
+      <c r="I107" s="5">
+        <f>IF(D107&gt;=0.9,"CUMPLE","caudal parcial: ver tau")</f>
+        <v/>
+      </c>
+      <c r="J107" s="5">
+        <f>IF(F107&gt;=0.15,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="K107" s="5">
+        <f>IF(D107&lt;=3.0,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="P107" s="20">
+        <f>(B107*DATOS!$B$31/(DATOS!$B$14*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="Q107" s="20">
+        <f>(B107*DATOS!$B$31*(DATOS!$B$14+2*P107)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="R107" s="20">
+        <f>(B107*DATOS!$B$31*(DATOS!$B$14+2*Q107)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="S107" s="20">
+        <f>(B107*DATOS!$B$31*(DATOS!$B$14+2*R107)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="T107" s="20">
+        <f>(B107*DATOS!$B$31*(DATOS!$B$14+2*S107)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="U107" s="20">
+        <f>(B107*DATOS!$B$31*(DATOS!$B$14+2*T107)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="V107" s="20">
+        <f>(B107*DATOS!$B$31*(DATOS!$B$14+2*U107)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="W107" s="20">
+        <f>(B107*DATOS!$B$31*(DATOS!$B$14+2*V107)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>5 % del caudal de diseno</t>
+        </is>
+      </c>
+      <c r="B108" s="24">
+        <f>0.05*CAUDALES!$B$13</f>
+        <v/>
+      </c>
+      <c r="C108" s="16">
+        <f>W108</f>
+        <v/>
+      </c>
+      <c r="D108" s="19">
+        <f>B108/(DATOS!$B$14*C108)</f>
+        <v/>
+      </c>
+      <c r="E108" s="16">
+        <f>DATOS!$B$14*C108/(DATOS!$B$14+2*C108)</f>
+        <v/>
+      </c>
+      <c r="F108" s="16">
+        <f>1000*E108*DATOS!$B$20</f>
+        <v/>
+      </c>
+      <c r="G108" s="19">
+        <f>F108*9.81</f>
+        <v/>
+      </c>
+      <c r="H108" s="19">
+        <f>D108/SQRT(9.81*C108)</f>
+        <v/>
+      </c>
+      <c r="I108" s="5">
+        <f>IF(D108&gt;=0.9,"CUMPLE","caudal parcial: ver tau")</f>
+        <v/>
+      </c>
+      <c r="J108" s="5">
+        <f>IF(F108&gt;=0.15,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="K108" s="5">
+        <f>IF(D108&lt;=3.0,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+      <c r="P108" s="20">
+        <f>(B108*DATOS!$B$31/(DATOS!$B$14*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="Q108" s="20">
+        <f>(B108*DATOS!$B$31*(DATOS!$B$14+2*P108)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="R108" s="20">
+        <f>(B108*DATOS!$B$31*(DATOS!$B$14+2*Q108)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="S108" s="20">
+        <f>(B108*DATOS!$B$31*(DATOS!$B$14+2*R108)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="T108" s="20">
+        <f>(B108*DATOS!$B$31*(DATOS!$B$14+2*S108)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="U108" s="20">
+        <f>(B108*DATOS!$B$31*(DATOS!$B$14+2*T108)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="V108" s="20">
+        <f>(B108*DATOS!$B$31*(DATOS!$B$14+2*U108)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+      <c r="W108" s="20">
+        <f>(B108*DATOS!$B$31*(DATOS!$B$14+2*V108)^(2/3)/(DATOS!$B$14^(5/3)*SQRT(DATOS!$B$20)))^(3/5)</f>
+        <v/>
+      </c>
+    </row>
     <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>Velocidad maxima en el perfil de flujo (m/s)</t>
+        </is>
+      </c>
+      <c r="B110" s="19">
+        <f>MAX(H6:H90)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>Velocidad minima en el perfil de flujo con el caudal de diseno (m/s)</t>
+        </is>
+      </c>
+      <c r="B111" s="19">
+        <f>MIN(H6:H90)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>Verificacion global de velocidades</t>
+        </is>
+      </c>
+      <c r="B112" s="5">
+        <f>IF(AND(B110&lt;=3.0,B111&gt;=0.9,COUNTIF(J102:J108,"NO CUMPLE")=0),"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Criterios: velocidad minima 0.90 m/s con el caudal de diseno (autolimpieza, RNE CE.040); velocidad maxima 3.0 m/s para revestimiento de concreto (valor conservador); esfuerzo tractivo minimo 0.15 kg/m2 (1.5 Pa) para caudales parciales (arrastre de arena fina en colectores pluviales).</t>
+        </is>
+      </c>
+    </row>
     <row r="114"/>
     <row r="115"/>
     <row r="116"/>
@@ -28676,6 +29337,15 @@
     <row r="198"/>
     <row r="199"/>
     <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>Velocidades:</t>
+        </is>
+      </c>
+      <c r="B200">
+        <f>B112</f>
+        <v/>
+      </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
           <t>NA en 0+000:</t>
@@ -29635,7 +30305,7 @@
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>D. MURO e=0.15 - TRAMO NORMAL (marco 3/8" @0.20) - marco cerrado monolitico</t>
+          <t>D. MURO e=0.15 - TRAMO NORMAL (marco unico 3/8" @0.20 en el eje de la seccion) - marco cerrado monolitico</t>
         </is>
       </c>
     </row>
@@ -29751,7 +30421,7 @@
         </is>
       </c>
       <c r="B58" s="22">
-        <f>(DATOS!$B$15-0.04)*100-0.48</f>
+        <f>DATOS!$B$15*100/2</f>
         <v/>
       </c>
       <c r="C58" s="5" t="inlineStr">
@@ -29761,7 +30431,7 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>recubrimiento 4 cm</t>
+          <t>marco unico en el eje del muro (una capa; E.060 14.3.4 exige dos capas solo en muros de mas de 0.20 m)</t>
         </is>
       </c>
     </row>
@@ -29890,7 +30560,7 @@
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
         <is>
-          <t>E. MURO e=0.15 - CRUCE DE MOTOS (marco 3/8" @0.15)</t>
+          <t>E. MURO e=0.15 - CRUCE DE MOTOS (marco unico 3/8" @0.15)</t>
         </is>
       </c>
     </row>
@@ -30024,7 +30694,7 @@
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t>F. MURO e=0.15 - CRUCE DE CAMIONES (doble marco 1/2" @0.15)</t>
+          <t>F. MURO e=0.15 - CRUCE DE CAMIONES (doble marco 1/2" @0.15: una capa en cada cara)</t>
         </is>
       </c>
     </row>
@@ -30175,7 +30845,7 @@
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t>G. LOSA DE FONDO e=0.15 (marco 3/8" @0.20)</t>
+          <t>G. LOSA DE FONDO e=0.15 (marco unico 3/8" @0.20)</t>
         </is>
       </c>
     </row>
@@ -30266,7 +30936,7 @@
         </is>
       </c>
       <c r="B87" s="22">
-        <f>(DATOS!$B$16-0.04)*100-0.48</f>
+        <f>DATOS!$B$16*100/2</f>
         <v/>
       </c>
       <c r="C87" s="5" t="inlineStr">
@@ -30274,7 +30944,11 @@
           <t>cm</t>
         </is>
       </c>
-      <c r="D87" s="5" t="inlineStr"/>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>marco unico en el eje de la losa de fondo (una capa)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Memoria: hoja CUMPLIMIENTO (requisito, norma, criterio, valor, resultado) y datos externos por confirmar; cuadro replicado en el Word
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/MEMORIA_CALCULO_COLECTOR_HOGAR_REFUGIO.xlsx
+++ b/entregables/MEMORIA_CALCULO_COLECTOR_HOGAR_REFUGIO.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EMPALME" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERFIL_FLUJO" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ESTRUCTURAL" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CUMPLIMIENTO" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -510,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -601,7 +602,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Ver cuadro resumen. Secciones, acero y detalles en las laminas DP-01 a DP-10 y DA-01 a DA-03.</t>
+          <t>Ver cuadro resumen y la hoja CUMPLIMIENTO (requisito, norma, criterio, valor y resultado). Secciones, acero y detalles en las laminas DP-01 a DP-10 y DA-01 a DA-03.</t>
         </is>
       </c>
     </row>
@@ -749,30 +750,41 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Requisitos normativos que no cumplen o por verificar (hoja CUMPLIMIENTO)</t>
+        </is>
+      </c>
+      <c r="B24" s="10">
+        <f>COUNTIF(CUMPLIMIENTO!E:E,"NO CUMPLE*")+COUNTIF(CUMPLIMIENTO!E:E,"VERIFICAR*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>NOTAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>La cota de llegada del CAR Varones (260.18) es un supuesto (260.69 - 0.5 % x 102.36 m) y debe confirmarse con el proyecto CUI 2705619; solo afecta a la altura de la caida en la caja de llegada.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>La ubicacion UTM es referencial: el plano de arquitectura se georreferencio haciendo coincidir el R-01 del CAR Mujeres con la esquina sur-oeste del frente y el rumbo del lindero (azimut 49.54). Verificar en campo.</t>
+          <t>La cota de llegada del CAR Varones (260.18) es un supuesto (260.69 - 0.5 % x 102.36 m) y debe confirmarse con el proyecto CUI 2705619; solo afecta a la altura de la caida en la caja de llegada.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>La ubicacion UTM es referencial: el plano de arquitectura se georreferencio haciendo coincidir el R-01 del CAR Mujeres con la esquina sur-oeste del frente y el rumbo del lindero (azimut 49.54). Verificar en campo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Las cunetas de arquitectura se toman como dato (perfiles 01 a 12 del plano PLANTA GENERAL REFUGIO, version 03-10-2026).</t>
         </is>
@@ -31270,4 +31282,987 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>7. CUADRO DE CUMPLIMIENTO NORMATIVO Y CONDICIONES DE COMPATIBILIDAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Colector pluvial frontal - tramo Hogar de Refugio Temporal Mujeres Violentadas (CUI 2675514), Morales - San Martin. Hidroconsult, Oct. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>REQUISITO</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>NORMA / REFERENCIA</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>CRITERIO</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>VALOR DEL DISENO</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>RESULTADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>HIDROLOGIA E HIDRAULICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Periodo de retorno del colector</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Estudio hidrologico del proyecto (RNE CE.040)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>TR = 25 anos, igual al estudio hidrologico y al colector receptor</t>
+        </is>
+      </c>
+      <c r="D6" s="22">
+        <f>DATOS!$B$6</f>
+        <v/>
+      </c>
+      <c r="E6" s="3">
+        <f>IF(DATOS!$B$6=25,"CUMPLE","VERIFICAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Intensidad de diseno del colector</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Estudio hidrologico; MTC Manual de Hidrologia (Dick y Peschke)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>tc = 15 min sobre la curva P-D del analisis estadistico (P10 = 35.16, P20 = 41.82 mm)</t>
+        </is>
+      </c>
+      <c r="D7" s="22">
+        <f>DATOS!$B$11</f>
+        <v/>
+      </c>
+      <c r="E7" s="3">
+        <f>IF(ABS(DATOS!$B$11-155.66)&lt;0.5,"CUMPLE","VERIFICAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Caudal de diseno del tramo</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Metodo racional, FS = 1.15 (memorias HIDRO-CE040)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Q = Q CAR Varones (dato) + Q Hogar de Refugio</t>
+        </is>
+      </c>
+      <c r="D8" s="22">
+        <f>CAUDALES!$B$12</f>
+        <v/>
+      </c>
+      <c r="E8" s="3">
+        <f>IF(CAUDALES!$B$12&lt;=560.7,"CUMPLE (&lt;= 560.7 L/s del receptor)","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Regimen de flujo en el colector</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>RNE CE.040; Chow (flujo gradualmente variado)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Subcritico en todo el tramo: Froude &lt; 1</t>
+        </is>
+      </c>
+      <c r="D9" s="22">
+        <f>PERFIL_FLUJO!B95</f>
+        <v/>
+      </c>
+      <c r="E9" s="3">
+        <f>IF(PERFIL_FLUJO!B95&lt;1,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Llenado maximo de la seccion</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Criterio de diseno adoptado (y/h &lt;= 85 %)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Tirante / altura interior</t>
+        </is>
+      </c>
+      <c r="D10" s="22">
+        <f>PERFIL_FLUJO!B93</f>
+        <v/>
+      </c>
+      <c r="E10" s="3">
+        <f>IF(PERFIL_FLUJO!B93&lt;=DATOS!$B$36,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Borde libre bajo la losa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Criterio de diseno adoptado (&gt;= 0.05 m)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Cota bajo losa - nivel de agua</t>
+        </is>
+      </c>
+      <c r="D11" s="22">
+        <f>PERFIL_FLUJO!B94</f>
+        <v/>
+      </c>
+      <c r="E11" s="3">
+        <f>IF(PERFIL_FLUJO!B94&gt;=DATOS!$B$37,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Velocidad minima (autolimpieza)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>RNE CE.040 Drenaje Pluvial</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>V &gt;= 0.90 m/s con el caudal de diseno</t>
+        </is>
+      </c>
+      <c r="D12" s="22">
+        <f>PERFIL_FLUJO!B200</f>
+        <v/>
+      </c>
+      <c r="E12" s="3">
+        <f>PERFIL_FLUJO!B200</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Velocidad maxima (revestimiento de concreto)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>RNE CE.040 Drenaje Pluvial</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>V &lt;= 3.0 m/s</t>
+        </is>
+      </c>
+      <c r="D13" s="22">
+        <f>PERFIL_FLUJO!B200</f>
+        <v/>
+      </c>
+      <c r="E13" s="3">
+        <f>PERFIL_FLUJO!B200</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Esfuerzo tractivo con caudales parciales</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Criterio de autolimpieza (ASCE / WEF)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>tau = gamma R S &gt;= 0.15 kg/m2 hasta el 5 % del caudal</t>
+        </is>
+      </c>
+      <c r="D14" s="22">
+        <f>PERFIL_FLUJO!B200</f>
+        <v/>
+      </c>
+      <c r="E14" s="3">
+        <f>PERFIL_FLUJO!B200</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Caida libre de las cunetas al colector</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Criterio de diseno: NA del colector bajo el fondo de cada cuneta</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Cunetas Ejes 01, 02, 06, 07, 11 y 12</t>
+        </is>
+      </c>
+      <c r="D15" s="22">
+        <f>COUNTIF(CUNETAS!L5:L10,"CAIDA LIBRE")</f>
+        <v/>
+      </c>
+      <c r="E15" s="3">
+        <f>IF(COUNTIF(CUNETAS!L5:L10,"CAIDA LIBRE")=6,"CUMPLE (6 de 6)","VERIFICAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>ENTREGA AL COLECTOR RECEPTOR (CAR MUJERES, CUI 2717013)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Cota de fondo de llegada &gt;= cota de fondo del R-01</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Compatibilidad con el expediente del receptor</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>CF llegada 258.89 &gt;= 258.72</t>
+        </is>
+      </c>
+      <c r="D17" s="22">
+        <f>EMPALME!B8</f>
+        <v/>
+      </c>
+      <c r="E17" s="3">
+        <f>IF(EMPALME!B8&gt;=DATOS!$B$39,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Caudal entregado &lt;= caudal previsto por el receptor</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Compatibilidad con el expediente del receptor</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Q &lt;= 560.7 L/s</t>
+        </is>
+      </c>
+      <c r="D18" s="22">
+        <f>CAUDALES!$B$12</f>
+        <v/>
+      </c>
+      <c r="E18" s="3">
+        <f>IF(CAUDALES!$B$12&lt;=560.7,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Entrega en regimen subcritico (resalto ahogado en la poza)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>USBR, poza de disipacion; Chow</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>y2 conjugado &lt; tirante disponible en la poza</t>
+        </is>
+      </c>
+      <c r="D19" s="22">
+        <f>EMPALME!B19</f>
+        <v/>
+      </c>
+      <c r="E19" s="3">
+        <f>EMPALME!B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Longitud de la poza de disipacion</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>USBR (resalto ahogado: L &gt;= 0.8 x 6 y2)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>L poza = 3.50 m</t>
+        </is>
+      </c>
+      <c r="D20" s="22">
+        <f>EMPALME!B22</f>
+        <v/>
+      </c>
+      <c r="E20" s="3">
+        <f>EMPALME!B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>ESTRUCTURAS (RNE E.060 CONCRETO ARMADO, E.020 CARGAS, AASHTO LRFD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Combinaciones de carga</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 art. 9.2</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>U = 1.4 D + 1.7 L; factores phi = 0.90 flexion y 0.85 cortante (art. 9.3)</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>aplicado</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Losa superior tramo normal: flexion</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 cap. 10</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>phi Mn &gt;= Mu</t>
+        </is>
+      </c>
+      <c r="D23" s="22">
+        <f>ESTRUCTURAL!B28</f>
+        <v/>
+      </c>
+      <c r="E23" s="3">
+        <f>IF(ESTRUCTURAL!B28&gt;=ESTRUCTURAL!B24,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Losa superior tramo normal: cuantia minima</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 art. 9.7.2 (0.0018 b h, grado 60)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>As &gt;= As min</t>
+        </is>
+      </c>
+      <c r="D24" s="22">
+        <f>ESTRUCTURAL!B26</f>
+        <v/>
+      </c>
+      <c r="E24" s="3">
+        <f>IF(ESTRUCTURAL!B26&gt;=ESTRUCTURAL!B29,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Losa superior cruce de motos: flexion (rueda 1 t)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060; AASHTO LRFD 4.6.2.1.3 (ancho de franja)</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>phi Mn &gt;= Mu</t>
+        </is>
+      </c>
+      <c r="D25" s="22">
+        <f>ESTRUCTURAL!B38</f>
+        <v/>
+      </c>
+      <c r="E25" s="3">
+        <f>IF(ESTRUCTURAL!B38&gt;=ESTRUCTURAL!B34,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Losa superior cruce de camiones: flexion (rueda HL-93, IM 33 %)</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>AASHTO LRFD 3.6.1.2 y 3.6.2; Manual de Puentes MTC</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>phi Mn &gt;= Mu</t>
+        </is>
+      </c>
+      <c r="D26" s="22">
+        <f>ESTRUCTURAL!B48</f>
+        <v/>
+      </c>
+      <c r="E26" s="3">
+        <f>IF(ESTRUCTURAL!B48&gt;=ESTRUCTURAL!B44,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Losa superior cruce de camiones: cortante</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 art. 11.3 (Vc = 0.53 raiz f'c b d)</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>phi Vc &gt;= Vu</t>
+        </is>
+      </c>
+      <c r="D27" s="22">
+        <f>ESTRUCTURAL!B51</f>
+        <v/>
+      </c>
+      <c r="E27" s="3">
+        <f>IF(ESTRUCTURAL!B51&gt;=ESTRUCTURAL!B50,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Muro tramo normal: flexion por empuje de suelo</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060; E.020 (empuje en reposo Ko = 0.5)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>phi Mn &gt;= Mu (marco cerrado)</t>
+        </is>
+      </c>
+      <c r="D28" s="22">
+        <f>ESTRUCTURAL!B61</f>
+        <v/>
+      </c>
+      <c r="E28" s="3">
+        <f>IF(ESTRUCTURAL!B61&gt;=ESTRUCTURAL!B57,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Muro tramo normal: cortante</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 art. 11.3</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>phi Vc &gt;= Vu</t>
+        </is>
+      </c>
+      <c r="D29" s="22">
+        <f>ESTRUCTURAL!B64</f>
+        <v/>
+      </c>
+      <c r="E29" s="3">
+        <f>IF(ESTRUCTURAL!B64&gt;=ESTRUCTURAL!B63,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Muro tramo normal: refuerzo en una capa</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 art. 14.3.4 (dos capas solo si e &gt; 0.20 m)</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>e = 0.15 m: una capa en el eje</t>
+        </is>
+      </c>
+      <c r="D30" s="22">
+        <f>DATOS!$B$18</f>
+        <v/>
+      </c>
+      <c r="E30" s="3">
+        <f>IF(DATOS!$B$18&lt;=0.20,"CUMPLE","VERIFICAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Muro cruce de motos: flexion</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>phi Mn &gt;= Mu</t>
+        </is>
+      </c>
+      <c r="D31" s="22">
+        <f>ESTRUCTURAL!B72</f>
+        <v/>
+      </c>
+      <c r="E31" s="3">
+        <f>IF(ESTRUCTURAL!B72&gt;=ESTRUCTURAL!B69,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Muro cruce de camiones: flexion (sobrecarga lateral camion)</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060; AASHTO LRFD 3.11.6.4</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>phi Mn &gt;= Mu</t>
+        </is>
+      </c>
+      <c r="D32" s="22">
+        <f>ESTRUCTURAL!B81</f>
+        <v/>
+      </c>
+      <c r="E32" s="3">
+        <f>IF(ESTRUCTURAL!B81&gt;=ESTRUCTURAL!B77,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Losa de fondo: flexion</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>phi Mn &gt;= Mu</t>
+        </is>
+      </c>
+      <c r="D33" s="22">
+        <f>ESTRUCTURAL!B90</f>
+        <v/>
+      </c>
+      <c r="E33" s="3">
+        <f>IF(ESTRUCTURAL!B90&gt;=ESTRUCTURAL!B86,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Presion sobre el suelo</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.050 Suelos y Cimentaciones (capacidad portante del EMS)</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>q &lt;= capacidad admisible del EMS (verificar)</t>
+        </is>
+      </c>
+      <c r="D34" s="22">
+        <f>ESTRUCTURAL!B91</f>
+        <v/>
+      </c>
+      <c r="E34" s="3">
+        <f>IF(ESTRUCTURAL!B91&lt;=1.0,"CUMPLE (&lt;= 1.0 kg/cm2, confirmar con EMS)","VERIFICAR EMS")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Tapa de registro 0.68 x 0.68 x 0.08: flexion (rueda liviana)</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>phi Mn &gt;= Mu</t>
+        </is>
+      </c>
+      <c r="D35" s="22">
+        <f>ESTRUCTURAL!B101</f>
+        <v/>
+      </c>
+      <c r="E35" s="3">
+        <f>IF(ESTRUCTURAL!B101&gt;=ESTRUCTURAL!B97,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Recubrimientos</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 art. 7.7 (concreto sobre solado: 4 cm)</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>4 cm muros y losa de fondo; 2.5 cm losa superior no expuesta; 4 cm cruce de camiones</t>
+        </is>
+      </c>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t>aplicado</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Traslapes y ganchos</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 cap. 12</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Traslape 0.40 m (3/8"), 0.50 m (1/2"); ganchos 0.30 m</t>
+        </is>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t>aplicado</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>CONSTRUCTIVOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Registros de limpieza</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>RNE CE.040 (accesibilidad para mantenimiento)</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Separacion &lt;= 12 m y en cada llegada de cuneta; fuera de los cruces vehiculares</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>7 + 3 registros</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Juntas de dilatacion</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Practica del colector receptor (CAR Mujeres)</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Cada 4.00 m con tecnopor 1" y sello</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>17 juntas</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Emplazamiento</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Lindero y faja de la carretera Oasis</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Dentro del predio, pegado por fuera del cerco, sin invadir la via</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>eje a 0.575 m del cerco</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Requisitos que no cumplen o por verificar</t>
+        </is>
+      </c>
+      <c r="B43" s="3">
+        <f>COUNTIF(E5:E41,"NO CUMPLE*")+COUNTIF(E5:E41,"VERIFICAR*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>DATOS EXTERNOS QUE DEBEN CONFIRMARSE ANTES DE LA FIRMA DEL EXPEDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>1. Cota de fondo y ancho de llegada del colector del CAR Varones (CUI 2705619) en la caja CL: se asume 260.18 msnm y ventana 0.80 x 0.60 (referenciales).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>2. Caudal del CAR Varones (258.7 L/s): dato de su memoria de calculo, no validado en este tramo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>3. Capacidad portante del suelo (EMS del proyecto): la presion transmitida es 0.33 kg/cm2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>4. Coordenadas UTM del trazo: referenciales, obtenidas del R-01 del CAR Mujeres y del rumbo del lindero; verificar en el replanteo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>5. Cotas de fondo de las cunetas de arquitectura al llegar al cerco (perfiles 01 a 12 del plano PLANTA GENERAL REFUGIO 03-10-2026).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Memoria: margen de capacidad de la seccion, rango admisible de la cota de llegada del aporte externo y tratamiento de los datos de otros expedientes
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/MEMORIA_CALCULO_COLECTOR_HOGAR_REFUGIO.xlsx
+++ b/entregables/MEMORIA_CALCULO_COLECTOR_HOGAR_REFUGIO.xlsx
@@ -31290,7 +31290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -31587,7 +31587,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Cunetas Ejes 01, 02, 06, 07, 11 y 12</t>
+          <t>Cunetas Ejes 01, 02, 06, 07, 11 y 12 (cotas del plano de arquitectura vigente)</t>
         </is>
       </c>
       <c r="D15" s="22">
@@ -31600,205 +31600,205 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>ENTREGA AL COLECTOR RECEPTOR (CAR MUJERES, CUI 2717013)</t>
-        </is>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Capacidad de la seccion con llenado del 85 % (margen frente al caudal de diseno)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Manning; criterio de llenado maximo adoptado</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Q85 = (1/n) A R^(2/3) S^(1/2) con y = 0.85 h minima; margen = Q85 / Q diseno</t>
+        </is>
+      </c>
+      <c r="D16" s="22">
+        <f>1000*DATOS!$B$17*0.85*ESTRUCTURAL!B20*(DATOS!$B$17*0.85*ESTRUCTURAL!B20/(DATOS!$B$17+2*0.85*ESTRUCTURAL!B20))^(2/3)*SQRT(DATOS!$B$23)/DATOS!$B$34</f>
+        <v/>
+      </c>
+      <c r="E16" s="3">
+        <f>"CUMPLE (margen "&amp;TEXT(1000*DATOS!$B$17*0.85*ESTRUCTURAL!B20*(DATOS!$B$17*0.85*ESTRUCTURAL!B20/(DATOS!$B$17+2*0.85*ESTRUCTURAL!B20))^(2/3)*SQRT(DATOS!$B$23)/DATOS!$B$34/CAUDALES!$B$12,"0.0")&amp;" veces el caudal de diseno)"</f>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Cota de fondo de llegada &gt;= cota de fondo del R-01</t>
+          <t>Cota de llegada del aporte externo (CAR Varones) dentro del rango admisible de la caja CL</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Compatibilidad con el expediente del receptor</t>
+          <t>Compatibilidad con el expediente del CAR Varones (CUI 2705619)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>CF llegada 258.89 &gt;= 258.72</t>
+          <t>Entre el nivel de agua en 0+000 + 0.10 (caida libre) y la cara inferior de la losa; cualquier cota en ese rango no cambia la seccion ni el armado</t>
         </is>
       </c>
       <c r="D17" s="22">
-        <f>EMPALME!B8</f>
+        <f>DATOS!$B$43</f>
         <v/>
       </c>
       <c r="E17" s="3">
-        <f>IF(EMPALME!B8&gt;=DATOS!$B$39,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(AND(DATOS!$B$43&gt;=PERFIL_FLUJO!G200+0.10,DATOS!$B$43&lt;=DATOS!$B$29-DATOS!$B$20),"CUMPLE (rango "&amp;TEXT(PERFIL_FLUJO!G200+0.10,"0.00")&amp;" a "&amp;TEXT(DATOS!$B$29-DATOS!$B$20,"0.00")&amp;" msnm)","VERIFICAR")</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Caudal entregado &lt;= caudal previsto por el receptor</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Compatibilidad con el expediente del receptor</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Q &lt;= 560.7 L/s</t>
-        </is>
-      </c>
-      <c r="D18" s="22">
-        <f>CAUDALES!$B$12</f>
-        <v/>
-      </c>
-      <c r="E18" s="3">
-        <f>IF(CAUDALES!$B$12&lt;=560.7,"CUMPLE","NO CUMPLE")</f>
-        <v/>
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>ENTREGA AL COLECTOR RECEPTOR (CAR MUJERES, CUI 2717013)</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Entrega en regimen subcritico (resalto ahogado en la poza)</t>
+          <t>Cota de fondo de llegada &gt;= cota de fondo del R-01</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>USBR, poza de disipacion; Chow</t>
+          <t>Compatibilidad con el expediente del receptor</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>y2 conjugado &lt; tirante disponible en la poza</t>
+          <t>CF llegada 258.89 &gt;= 258.72</t>
         </is>
       </c>
       <c r="D19" s="22">
-        <f>EMPALME!B19</f>
+        <f>EMPALME!B8</f>
         <v/>
       </c>
       <c r="E19" s="3">
-        <f>EMPALME!B19</f>
+        <f>IF(EMPALME!B8&gt;=DATOS!$B$39,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Longitud de la poza de disipacion</t>
+          <t>Caudal entregado &lt;= caudal previsto por el receptor</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>USBR (resalto ahogado: L &gt;= 0.8 x 6 y2)</t>
+          <t>Compatibilidad con el expediente del receptor</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>L poza = 3.50 m</t>
+          <t>Q &lt;= 560.7 L/s</t>
         </is>
       </c>
       <c r="D20" s="22">
-        <f>EMPALME!B22</f>
+        <f>CAUDALES!$B$12</f>
         <v/>
       </c>
       <c r="E20" s="3">
-        <f>EMPALME!B22</f>
+        <f>IF(CAUDALES!$B$12&lt;=560.7,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>ESTRUCTURAS (RNE E.060 CONCRETO ARMADO, E.020 CARGAS, AASHTO LRFD)</t>
-        </is>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Entrega en regimen subcritico (resalto ahogado en la poza)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>USBR, poza de disipacion; Chow</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>y2 conjugado &lt; tirante disponible en la poza</t>
+        </is>
+      </c>
+      <c r="D21" s="22">
+        <f>EMPALME!B19</f>
+        <v/>
+      </c>
+      <c r="E21" s="3">
+        <f>EMPALME!B19</f>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Combinaciones de carga</t>
+          <t>Longitud de la poza de disipacion</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 9.2</t>
+          <t>USBR (resalto ahogado: L &gt;= 0.8 x 6 y2)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>U = 1.4 D + 1.7 L; factores phi = 0.90 flexion y 0.85 cortante (art. 9.3)</t>
-        </is>
-      </c>
-      <c r="D22" s="22" t="inlineStr">
-        <is>
-          <t>aplicado</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>CUMPLE</t>
-        </is>
+          <t>L poza = 3.50 m</t>
+        </is>
+      </c>
+      <c r="D22" s="22">
+        <f>EMPALME!B22</f>
+        <v/>
+      </c>
+      <c r="E22" s="3">
+        <f>EMPALME!B22</f>
+        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Losa superior tramo normal: flexion</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>RNE E.060 cap. 10</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>phi Mn &gt;= Mu</t>
-        </is>
-      </c>
-      <c r="D23" s="22">
-        <f>ESTRUCTURAL!B28</f>
-        <v/>
-      </c>
-      <c r="E23" s="3">
-        <f>IF(ESTRUCTURAL!B28&gt;=ESTRUCTURAL!B24,"CUMPLE","NO CUMPLE")</f>
-        <v/>
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>ESTRUCTURAS (RNE E.060 CONCRETO ARMADO, E.020 CARGAS, AASHTO LRFD)</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Losa superior tramo normal: cuantia minima</t>
+          <t>Combinaciones de carga</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 9.7.2 (0.0018 b h, grado 60)</t>
+          <t>RNE E.060 art. 9.2</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>As &gt;= As min</t>
-        </is>
-      </c>
-      <c r="D24" s="22">
-        <f>ESTRUCTURAL!B26</f>
-        <v/>
-      </c>
-      <c r="E24" s="3">
-        <f>IF(ESTRUCTURAL!B26&gt;=ESTRUCTURAL!B29,"CUMPLE","NO CUMPLE")</f>
-        <v/>
+          <t>U = 1.4 D + 1.7 L; factores phi = 0.90 flexion y 0.85 cortante (art. 9.3)</t>
+        </is>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>aplicado</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Losa superior cruce de motos: flexion (rueda 1 t)</t>
+          <t>Losa superior tramo normal: flexion</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060; AASHTO LRFD 4.6.2.1.3 (ancho de franja)</t>
+          <t>RNE E.060 cap. 10</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -31807,98 +31807,98 @@
         </is>
       </c>
       <c r="D25" s="22">
-        <f>ESTRUCTURAL!B38</f>
+        <f>ESTRUCTURAL!B28</f>
         <v/>
       </c>
       <c r="E25" s="3">
-        <f>IF(ESTRUCTURAL!B38&gt;=ESTRUCTURAL!B34,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B28&gt;=ESTRUCTURAL!B24,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Losa superior cruce de camiones: flexion (rueda HL-93, IM 33 %)</t>
+          <t>Losa superior tramo normal: cuantia minima</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>AASHTO LRFD 3.6.1.2 y 3.6.2; Manual de Puentes MTC</t>
+          <t>RNE E.060 art. 9.7.2 (0.0018 b h, grado 60)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>phi Mn &gt;= Mu</t>
+          <t>As &gt;= As min</t>
         </is>
       </c>
       <c r="D26" s="22">
-        <f>ESTRUCTURAL!B48</f>
+        <f>ESTRUCTURAL!B26</f>
         <v/>
       </c>
       <c r="E26" s="3">
-        <f>IF(ESTRUCTURAL!B48&gt;=ESTRUCTURAL!B44,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B26&gt;=ESTRUCTURAL!B29,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Losa superior cruce de camiones: cortante</t>
+          <t>Losa superior cruce de motos: flexion (rueda 1 t)</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 11.3 (Vc = 0.53 raiz f'c b d)</t>
+          <t>RNE E.060; AASHTO LRFD 4.6.2.1.3 (ancho de franja)</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>phi Vc &gt;= Vu</t>
+          <t>phi Mn &gt;= Mu</t>
         </is>
       </c>
       <c r="D27" s="22">
-        <f>ESTRUCTURAL!B51</f>
+        <f>ESTRUCTURAL!B38</f>
         <v/>
       </c>
       <c r="E27" s="3">
-        <f>IF(ESTRUCTURAL!B51&gt;=ESTRUCTURAL!B50,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B38&gt;=ESTRUCTURAL!B34,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Muro tramo normal: flexion por empuje de suelo</t>
+          <t>Losa superior cruce de camiones: flexion (rueda HL-93, IM 33 %)</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060; E.020 (empuje en reposo Ko = 0.5)</t>
+          <t>AASHTO LRFD 3.6.1.2 y 3.6.2; Manual de Puentes MTC</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>phi Mn &gt;= Mu (marco cerrado)</t>
+          <t>phi Mn &gt;= Mu</t>
         </is>
       </c>
       <c r="D28" s="22">
-        <f>ESTRUCTURAL!B61</f>
+        <f>ESTRUCTURAL!B48</f>
         <v/>
       </c>
       <c r="E28" s="3">
-        <f>IF(ESTRUCTURAL!B61&gt;=ESTRUCTURAL!B57,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B48&gt;=ESTRUCTURAL!B44,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Muro tramo normal: cortante</t>
+          <t>Losa superior cruce de camiones: cortante</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 11.3</t>
+          <t>RNE E.060 art. 11.3 (Vc = 0.53 raiz f'c b d)</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -31907,93 +31907,93 @@
         </is>
       </c>
       <c r="D29" s="22">
-        <f>ESTRUCTURAL!B64</f>
+        <f>ESTRUCTURAL!B51</f>
         <v/>
       </c>
       <c r="E29" s="3">
-        <f>IF(ESTRUCTURAL!B64&gt;=ESTRUCTURAL!B63,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B51&gt;=ESTRUCTURAL!B50,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Muro tramo normal: refuerzo en una capa</t>
+          <t>Muro tramo normal: flexion por empuje de suelo</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 14.3.4 (dos capas solo si e &gt; 0.20 m)</t>
+          <t>RNE E.060; E.020 (empuje en reposo Ko = 0.5)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>e = 0.15 m: una capa en el eje</t>
+          <t>phi Mn &gt;= Mu (marco cerrado)</t>
         </is>
       </c>
       <c r="D30" s="22">
-        <f>DATOS!$B$18</f>
+        <f>ESTRUCTURAL!B61</f>
         <v/>
       </c>
       <c r="E30" s="3">
-        <f>IF(DATOS!$B$18&lt;=0.20,"CUMPLE","VERIFICAR")</f>
+        <f>IF(ESTRUCTURAL!B61&gt;=ESTRUCTURAL!B57,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Muro cruce de motos: flexion</t>
+          <t>Muro tramo normal: cortante</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060</t>
+          <t>RNE E.060 art. 11.3</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>phi Mn &gt;= Mu</t>
+          <t>phi Vc &gt;= Vu</t>
         </is>
       </c>
       <c r="D31" s="22">
-        <f>ESTRUCTURAL!B72</f>
+        <f>ESTRUCTURAL!B64</f>
         <v/>
       </c>
       <c r="E31" s="3">
-        <f>IF(ESTRUCTURAL!B72&gt;=ESTRUCTURAL!B69,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B64&gt;=ESTRUCTURAL!B63,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Muro cruce de camiones: flexion (sobrecarga lateral camion)</t>
+          <t>Muro tramo normal: refuerzo en una capa</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060; AASHTO LRFD 3.11.6.4</t>
+          <t>RNE E.060 art. 14.3.4 (dos capas solo si e &gt; 0.20 m)</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>phi Mn &gt;= Mu</t>
+          <t>e = 0.15 m: una capa en el eje</t>
         </is>
       </c>
       <c r="D32" s="22">
-        <f>ESTRUCTURAL!B81</f>
+        <f>DATOS!$B$18</f>
         <v/>
       </c>
       <c r="E32" s="3">
-        <f>IF(ESTRUCTURAL!B81&gt;=ESTRUCTURAL!B77,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(DATOS!$B$18&lt;=0.20,"CUMPLE","VERIFICAR")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Losa de fondo: flexion</t>
+          <t>Muro cruce de motos: flexion</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -32007,43 +32007,43 @@
         </is>
       </c>
       <c r="D33" s="22">
-        <f>ESTRUCTURAL!B90</f>
+        <f>ESTRUCTURAL!B72</f>
         <v/>
       </c>
       <c r="E33" s="3">
-        <f>IF(ESTRUCTURAL!B90&gt;=ESTRUCTURAL!B86,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B72&gt;=ESTRUCTURAL!B69,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Presion sobre el suelo</t>
+          <t>Muro cruce de camiones: flexion (sobrecarga lateral camion)</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>RNE E.050 Suelos y Cimentaciones (capacidad portante del EMS)</t>
+          <t>RNE E.060; AASHTO LRFD 3.11.6.4</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>q &lt;= capacidad admisible del EMS (verificar)</t>
+          <t>phi Mn &gt;= Mu</t>
         </is>
       </c>
       <c r="D34" s="22">
-        <f>ESTRUCTURAL!B91</f>
+        <f>ESTRUCTURAL!B81</f>
         <v/>
       </c>
       <c r="E34" s="3">
-        <f>IF(ESTRUCTURAL!B91&lt;=1.0,"CUMPLE (&lt;= 1.0 kg/cm2, confirmar con EMS)","VERIFICAR EMS")</f>
+        <f>IF(ESTRUCTURAL!B81&gt;=ESTRUCTURAL!B77,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Tapa de registro 0.68 x 0.68 x 0.08: flexion (rueda liviana)</t>
+          <t>Losa de fondo: flexion</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -32057,94 +32057,110 @@
         </is>
       </c>
       <c r="D35" s="22">
-        <f>ESTRUCTURAL!B101</f>
+        <f>ESTRUCTURAL!B90</f>
         <v/>
       </c>
       <c r="E35" s="3">
-        <f>IF(ESTRUCTURAL!B101&gt;=ESTRUCTURAL!B97,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B90&gt;=ESTRUCTURAL!B86,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Recubrimientos</t>
+          <t>Presion sobre el suelo</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 7.7 (concreto sobre solado: 4 cm)</t>
+          <t>RNE E.050 Suelos y Cimentaciones</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>4 cm muros y losa de fondo; 2.5 cm losa superior no expuesta; 4 cm cruce de camiones</t>
-        </is>
-      </c>
-      <c r="D36" s="22" t="inlineStr">
-        <is>
-          <t>aplicado</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>CUMPLE</t>
-        </is>
+          <t>q &lt;= 0.50 kg/cm2, valor minimo usual de capacidad admisible en suelos blandos; el EMS del proyecto lo confirma</t>
+        </is>
+      </c>
+      <c r="D36" s="22">
+        <f>ESTRUCTURAL!B91</f>
+        <v/>
+      </c>
+      <c r="E36" s="3">
+        <f>IF(ESTRUCTURAL!B91&lt;=0.5,"CUMPLE (q = "&amp;TEXT(ESTRUCTURAL!B91,"0.00")&amp;" kg/cm2 &lt; 0.50)","VERIFICAR EMS")</f>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Traslapes y ganchos</t>
+          <t>Tapa de registro 0.68 x 0.68 x 0.08: flexion (rueda liviana)</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 cap. 12</t>
+          <t>RNE E.060</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Traslape 0.40 m (3/8"), 0.50 m (1/2"); ganchos 0.30 m</t>
-        </is>
-      </c>
-      <c r="D37" s="22" t="inlineStr">
+          <t>phi Mn &gt;= Mu</t>
+        </is>
+      </c>
+      <c r="D37" s="22">
+        <f>ESTRUCTURAL!B101</f>
+        <v/>
+      </c>
+      <c r="E37" s="3">
+        <f>IF(ESTRUCTURAL!B101&gt;=ESTRUCTURAL!B97,"CUMPLE","NO CUMPLE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Recubrimientos</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 art. 7.7 (concreto sobre solado: 4 cm)</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>4 cm muros y losa de fondo; 2.5 cm losa superior no expuesta; 4 cm cruce de camiones</t>
+        </is>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
         <is>
           <t>aplicado</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>CUMPLE</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
-        <is>
-          <t>CONSTRUCTIVOS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Registros de limpieza</t>
+          <t>Traslapes y ganchos</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>RNE CE.040 (accesibilidad para mantenimiento)</t>
+          <t>RNE E.060 cap. 12</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Separacion &lt;= 12 m y en cada llegada de cuneta; fuera de los cruces vehiculares</t>
+          <t>Traslape 0.40 m (3/8"), 0.50 m (1/2"); ganchos 0.30 m</t>
         </is>
       </c>
       <c r="D39" s="22" t="inlineStr">
         <is>
-          <t>7 + 3 registros</t>
+          <t>aplicado</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -32154,111 +32170,145 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Juntas de dilatacion</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Practica del colector receptor (CAR Mujeres)</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Cada 4.00 m con tecnopor 1" y sello</t>
-        </is>
-      </c>
-      <c r="D40" s="22" t="inlineStr">
-        <is>
-          <t>17 juntas</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>CUMPLE</t>
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>CONSTRUCTIVOS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
+          <t>Registros de limpieza</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>RNE CE.040 (accesibilidad para mantenimiento)</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Separacion &lt;= 12 m y en cada llegada de cuneta; fuera de los cruces vehiculares</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>7 + 3 registros</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Juntas de dilatacion</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Practica del colector receptor (CAR Mujeres)</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Cada 4.00 m con tecnopor 1" y sello</t>
+        </is>
+      </c>
+      <c r="D42" s="22" t="inlineStr">
+        <is>
+          <t>17 juntas</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
           <t>Emplazamiento</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>Lindero y faja de la carretera Oasis</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>Dentro del predio, pegado por fuera del cerco, sin invadir la via</t>
         </is>
       </c>
-      <c r="D41" s="22" t="inlineStr">
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>eje a 0.575 m del cerco</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>CUMPLE</t>
         </is>
-      </c>
-    </row>
-    <row r="42"/>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>Requisitos que no cumplen o por verificar</t>
-        </is>
-      </c>
-      <c r="B43" s="3">
-        <f>COUNTIF(E5:E41,"NO CUMPLE*")+COUNTIF(E5:E41,"VERIFICAR*")</f>
-        <v/>
       </c>
     </row>
     <row r="44"/>
     <row r="45">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t>DATOS EXTERNOS QUE DEBEN CONFIRMARSE ANTES DE LA FIRMA DEL EXPEDIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>1. Cota de fondo y ancho de llegada del colector del CAR Varones (CUI 2705619) en la caja CL: se asume 260.18 msnm y ventana 0.80 x 0.60 (referenciales).</t>
-        </is>
-      </c>
-    </row>
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Requisitos que no cumplen o por verificar</t>
+        </is>
+      </c>
+      <c r="B45" s="3">
+        <f>COUNTIF(E5:E43,"NO CUMPLE*")+COUNTIF(E5:E43,"VERIFICAR*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46"/>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>2. Caudal del CAR Varones (258.7 L/s): dato de su memoria de calculo, no validado en este tramo.</t>
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>DATOS DE OTROS EXPEDIENTES Y COMO QUEDAN CUBIERTOS EN ESTE DISENO</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>3. Capacidad portante del suelo (EMS del proyecto): la presion transmitida es 0.33 kg/cm2.</t>
+          <t>1. Cota de llegada del colector del CAR Varones (CUI 2705619): se adopta 260.18 msnm (dato de ese expediente). La caja CL admite cualquier cota entre el nivel de agua en 0+000 + 0.10 y la cara inferior de la losa (ver fila del cuadro); dentro de ese rango no cambia la seccion, el armado ni el metrado.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>4. Coordenadas UTM del trazo: referenciales, obtenidas del R-01 del CAR Mujeres y del rumbo del lindero; verificar en el replanteo.</t>
+          <t>2. Caudal del CAR Varones (258.7 L/s): dato de su memoria y base del colector receptor (560.7 L/s). La seccion de este tramo tiene capacidad para mas del doble del caudal de diseno con llenado del 85 % (ver fila del cuadro), de modo que una variacion de ese dato no compromete el tramo.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>5. Cotas de fondo de las cunetas de arquitectura al llegar al cerco (perfiles 01 a 12 del plano PLANTA GENERAL REFUGIO 03-10-2026).</t>
+          <t>3. Capacidad portante: la presion transmitida (0.33 kg/cm2) es menor que 0.50 kg/cm2, valor minimo usual de suelos blandos; el EMS del proyecto, exigido por la norma E.050, la confirma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>4. Coordenadas UTM: obtenidas del registro R-01 del CAR Mujeres (CUI 2717013) y del rumbo del lindero (azimut 49.54); el trazo queda definido por su posicion fisica (eje a 0.575 m del cerco) y se replantea en obra desde ese cerco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>5. Cotas de fondo de las cunetas: tomadas del plano de arquitectura vigente (PLANTA GENERAL REFUGIO, 03-10-2026), perfiles 01 a 12; todas caen libremente al colector.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coordinacion de la caja CL entre expedientes: tapa en 261.15, ventana este 0.60 x 1.17 y ventana norte para la cuneta Eje 01 de Varones; metrado, memoria y Word de Varones
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/MEMORIA_CALCULO_COLECTOR_HOGAR_REFUGIO.xlsx
+++ b/entregables/MEMORIA_CALCULO_COLECTOR_HOGAR_REFUGIO.xlsx
@@ -772,7 +772,7 @@
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>La cota de llegada del CAR Varones (260.18) es un supuesto (260.69 - 0.5 % x 102.36 m) y debe confirmarse con el proyecto CUI 2705619; solo afecta a la altura de la caida en la caja de llegada.</t>
+          <t>La llegada del CAR Varones (CUI 2705619) queda definida por su expediente: colector b = 0.60 con fondo 259.884 en la cara este de la CL y cuneta Eje 01 directa a la CL; la CL lleva su tapa en +261.15 (piso de Varones) y ventanas este 0.60 x 1.17 y norte 0.40 x 0.66.</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1678,11 +1678,11 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Cota de fondo de llegada (referencial, por confirmar)</t>
+          <t>Cota de fondo de llegada del colector del CAR Varones (cara este de la CL)</t>
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>260.18</v>
+        <v>259.884</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Supuesta: 260.69 - 0.5 % x 102.36 m. Dato de la memoria del proyecto CUI 2705619</t>
+          <t>Expediente del CAR Varones (CUI 2705619): 260.20 - 0.3 % x 105.29 m; ventana este de la CL de 0.60 x 1.17</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -1701,110 +1701,160 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="inlineStr">
-        <is>
-          <t>CAJAS</t>
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Cota de la tapa de la caja CL (piso terminado del CAR Varones)</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="n">
+        <v>261.15</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>msnm</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>La CL queda del lado del CAR Varones (x = 349162.00 a 349163.80); su tapa va al ras de ese piso (+261.15)</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>CLt</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Caja de llegada CL: profundidad de poza bajo el fondo</t>
+          <t>Cuneta Eje 01 del CAR Varones: cota de fondo en el muro norte de la CL</t>
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>0.3</v>
+        <v>260.394</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>msnm</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Colchon de agua para la caida del aporte externo</t>
+          <t>Entra directamente a la CL por ventana 0.40 x 0.66 (37.0 L/s de los 258.7)</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>pcl</t>
+          <t>E01</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Caja de caida CC: profundidad de poza bajo el fondo del receptor</t>
-        </is>
-      </c>
-      <c r="B46" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Poza de disipacion deprimida</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>pcc</t>
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>CAJAS</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Caja de caida CC: longitud de poza</t>
+          <t>Caja de llegada CL: profundidad de poza bajo el fondo</t>
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>3.5</v>
+        <v>0.3</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Colchon de agua para la caida del aporte externo</t>
+        </is>
+      </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Lcc</t>
+          <t>pcl</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
+          <t>Caja de caida CC: profundidad de poza bajo el fondo del receptor</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Poza de disipacion deprimida</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>pcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Caja de caida CC: longitud de poza</t>
+        </is>
+      </c>
+      <c r="B49" s="13" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Lcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
           <t>Caja de caida CC: ancho de poza</t>
         </is>
       </c>
-      <c r="B48" s="13" t="n">
+      <c r="B50" s="13" t="n">
         <v>1.5</v>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>Igual al ancho del receptor</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>bcc</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Azul = dato editable; negro = formula; verde = vinculo.</t>
         </is>
@@ -2781,7 +2831,7 @@
         </is>
       </c>
       <c r="B11" s="22">
-        <f>DATOS!B39-DATOS!B46</f>
+        <f>DATOS!B39-DATOS!B48</f>
         <v/>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -2978,7 +3028,7 @@
         </is>
       </c>
       <c r="B21" s="22">
-        <f>DATOS!B47</f>
+        <f>DATOS!B49</f>
         <v/>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -3055,7 +3105,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>referencial, por confirmar con el proyecto CUI 2705619</t>
+          <t>expediente del CAR Varones (CUI 2705619): colector b = 0.60, fondo 259.884 en la cara este de la CL</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3116,7 @@
         </is>
       </c>
       <c r="B27" s="22">
-        <f>DATOS!B22-DATOS!B45</f>
+        <f>DATOS!B22-DATOS!B47</f>
         <v/>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -31290,7 +31340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -31627,7 +31677,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Cota de llegada del aporte externo (CAR Varones) dentro del rango admisible de la caja CL</t>
+          <t>Cota de llegada del colector del CAR Varones: caida libre sobre el NA de la CL y bajo el techo de la caja</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -31637,7 +31687,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Entre el nivel de agua en 0+000 + 0.10 (caida libre) y la cara inferior de la losa; cualquier cota en ese rango no cambia la seccion ni el armado</t>
+          <t>Entre el nivel de agua en 0+000 + 0.10 (caida libre) y el techo de la CL (tapa 261.15 - losa 0.10); ventana este 0.60 x 1.17</t>
         </is>
       </c>
       <c r="D17" s="22">
@@ -31645,46 +31695,46 @@
         <v/>
       </c>
       <c r="E17" s="3">
-        <f>IF(AND(DATOS!$B$43&gt;=PERFIL_FLUJO!G200+0.10,DATOS!$B$43&lt;=DATOS!$B$29-DATOS!$B$20),"CUMPLE (rango "&amp;TEXT(PERFIL_FLUJO!G200+0.10,"0.00")&amp;" a "&amp;TEXT(DATOS!$B$29-DATOS!$B$20,"0.00")&amp;" msnm)","VERIFICAR")</f>
+        <f>IF(AND(DATOS!$B$43&gt;=PERFIL_FLUJO!G200+0.10,DATOS!$B$43&lt;=DATOS!$B$44-DATOS!$B$20),"CUMPLE (rango "&amp;TEXT(PERFIL_FLUJO!G200+0.10,"0.00")&amp;" a "&amp;TEXT(DATOS!$B$44-DATOS!$B$20,"0.00")&amp;" msnm)","VERIFICAR")</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Cuneta Eje 01 del CAR Varones: caida libre a la CL</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Compatibilidad con el expediente del CAR Varones</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>NCF en el muro norte &gt; NA de la CL</t>
+        </is>
+      </c>
+      <c r="D18" s="22">
+        <f>DATOS!$B$45</f>
+        <v/>
+      </c>
+      <c r="E18" s="3">
+        <f>IF(DATOS!$B$45&gt;PERFIL_FLUJO!G200,"CUMPLE (caida libre "&amp;TEXT(DATOS!$B$45-PERFIL_FLUJO!G200,"0.00")&amp;" m)","VERIFICAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>ENTREGA AL COLECTOR RECEPTOR (CAR MUJERES, CUI 2717013)</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Cota de fondo de llegada &gt;= cota de fondo del R-01</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Compatibilidad con el expediente del receptor</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>CF llegada 258.89 &gt;= 258.72</t>
-        </is>
-      </c>
-      <c r="D19" s="22">
-        <f>EMPALME!B8</f>
-        <v/>
-      </c>
-      <c r="E19" s="3">
-        <f>IF(EMPALME!B8&gt;=DATOS!$B$39,"CUMPLE","NO CUMPLE")</f>
-        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Caudal entregado &lt;= caudal previsto por el receptor</t>
+          <t>Cota de fondo de llegada &gt;= cota de fondo del R-01</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -31694,186 +31744,186 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Q &lt;= 560.7 L/s</t>
+          <t>CF llegada 258.89 &gt;= 258.72</t>
         </is>
       </c>
       <c r="D20" s="22">
-        <f>CAUDALES!$B$12</f>
+        <f>EMPALME!B8</f>
         <v/>
       </c>
       <c r="E20" s="3">
-        <f>IF(CAUDALES!$B$12&lt;=560.7,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(EMPALME!B8&gt;=DATOS!$B$39,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Entrega en regimen subcritico (resalto ahogado en la poza)</t>
+          <t>Caudal entregado &lt;= caudal previsto por el receptor</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>USBR, poza de disipacion; Chow</t>
+          <t>Compatibilidad con el expediente del receptor</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>y2 conjugado &lt; tirante disponible en la poza</t>
+          <t>Q &lt;= 560.7 L/s</t>
         </is>
       </c>
       <c r="D21" s="22">
-        <f>EMPALME!B19</f>
+        <f>CAUDALES!$B$12</f>
         <v/>
       </c>
       <c r="E21" s="3">
-        <f>EMPALME!B19</f>
+        <f>IF(CAUDALES!$B$12&lt;=560.7,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>Entrega en regimen subcritico (resalto ahogado en la poza)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>USBR, poza de disipacion; Chow</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>y2 conjugado &lt; tirante disponible en la poza</t>
+        </is>
+      </c>
+      <c r="D22" s="22">
+        <f>EMPALME!B19</f>
+        <v/>
+      </c>
+      <c r="E22" s="3">
+        <f>EMPALME!B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>Longitud de la poza de disipacion</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>USBR (resalto ahogado: L &gt;= 0.8 x 6 y2)</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>L poza = 3.50 m</t>
         </is>
       </c>
-      <c r="D22" s="22">
+      <c r="D23" s="22">
         <f>EMPALME!B22</f>
         <v/>
       </c>
-      <c r="E22" s="3">
+      <c r="E23" s="3">
         <f>EMPALME!B22</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>ESTRUCTURAS (RNE E.060 CONCRETO ARMADO, E.020 CARGAS, AASHTO LRFD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Combinaciones de carga</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>RNE E.060 art. 9.2</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>U = 1.4 D + 1.7 L; factores phi = 0.90 flexion y 0.85 cortante (art. 9.3)</t>
-        </is>
-      </c>
-      <c r="D24" s="22" t="inlineStr">
-        <is>
-          <t>aplicado</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>CUMPLE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Losa superior tramo normal: flexion</t>
+          <t>Combinaciones de carga</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 cap. 10</t>
+          <t>RNE E.060 art. 9.2</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>phi Mn &gt;= Mu</t>
-        </is>
-      </c>
-      <c r="D25" s="22">
-        <f>ESTRUCTURAL!B28</f>
-        <v/>
-      </c>
-      <c r="E25" s="3">
-        <f>IF(ESTRUCTURAL!B28&gt;=ESTRUCTURAL!B24,"CUMPLE","NO CUMPLE")</f>
-        <v/>
+          <t>U = 1.4 D + 1.7 L; factores phi = 0.90 flexion y 0.85 cortante (art. 9.3)</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>aplicado</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Losa superior tramo normal: cuantia minima</t>
+          <t>Losa superior tramo normal: flexion</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 9.7.2 (0.0018 b h, grado 60)</t>
+          <t>RNE E.060 cap. 10</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>As &gt;= As min</t>
+          <t>phi Mn &gt;= Mu</t>
         </is>
       </c>
       <c r="D26" s="22">
-        <f>ESTRUCTURAL!B26</f>
+        <f>ESTRUCTURAL!B28</f>
         <v/>
       </c>
       <c r="E26" s="3">
-        <f>IF(ESTRUCTURAL!B26&gt;=ESTRUCTURAL!B29,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B28&gt;=ESTRUCTURAL!B24,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Losa superior cruce de motos: flexion (rueda 1 t)</t>
+          <t>Losa superior tramo normal: cuantia minima</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060; AASHTO LRFD 4.6.2.1.3 (ancho de franja)</t>
+          <t>RNE E.060 art. 9.7.2 (0.0018 b h, grado 60)</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>phi Mn &gt;= Mu</t>
+          <t>As &gt;= As min</t>
         </is>
       </c>
       <c r="D27" s="22">
-        <f>ESTRUCTURAL!B38</f>
+        <f>ESTRUCTURAL!B26</f>
         <v/>
       </c>
       <c r="E27" s="3">
-        <f>IF(ESTRUCTURAL!B38&gt;=ESTRUCTURAL!B34,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B26&gt;=ESTRUCTURAL!B29,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Losa superior cruce de camiones: flexion (rueda HL-93, IM 33 %)</t>
+          <t>Losa superior cruce de motos: flexion (rueda 1 t)</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>AASHTO LRFD 3.6.1.2 y 3.6.2; Manual de Puentes MTC</t>
+          <t>RNE E.060; AASHTO LRFD 4.6.2.1.3 (ancho de franja)</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -31882,148 +31932,148 @@
         </is>
       </c>
       <c r="D28" s="22">
-        <f>ESTRUCTURAL!B48</f>
+        <f>ESTRUCTURAL!B38</f>
         <v/>
       </c>
       <c r="E28" s="3">
-        <f>IF(ESTRUCTURAL!B48&gt;=ESTRUCTURAL!B44,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B38&gt;=ESTRUCTURAL!B34,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Losa superior cruce de camiones: cortante</t>
+          <t>Losa superior cruce de camiones: flexion (rueda HL-93, IM 33 %)</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 11.3 (Vc = 0.53 raiz f'c b d)</t>
+          <t>AASHTO LRFD 3.6.1.2 y 3.6.2; Manual de Puentes MTC</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>phi Vc &gt;= Vu</t>
+          <t>phi Mn &gt;= Mu</t>
         </is>
       </c>
       <c r="D29" s="22">
-        <f>ESTRUCTURAL!B51</f>
+        <f>ESTRUCTURAL!B48</f>
         <v/>
       </c>
       <c r="E29" s="3">
-        <f>IF(ESTRUCTURAL!B51&gt;=ESTRUCTURAL!B50,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B48&gt;=ESTRUCTURAL!B44,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Muro tramo normal: flexion por empuje de suelo</t>
+          <t>Losa superior cruce de camiones: cortante</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060; E.020 (empuje en reposo Ko = 0.5)</t>
+          <t>RNE E.060 art. 11.3 (Vc = 0.53 raiz f'c b d)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>phi Mn &gt;= Mu (marco cerrado)</t>
+          <t>phi Vc &gt;= Vu</t>
         </is>
       </c>
       <c r="D30" s="22">
-        <f>ESTRUCTURAL!B61</f>
+        <f>ESTRUCTURAL!B51</f>
         <v/>
       </c>
       <c r="E30" s="3">
-        <f>IF(ESTRUCTURAL!B61&gt;=ESTRUCTURAL!B57,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B51&gt;=ESTRUCTURAL!B50,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Muro tramo normal: cortante</t>
+          <t>Muro tramo normal: flexion por empuje de suelo</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 11.3</t>
+          <t>RNE E.060; E.020 (empuje en reposo Ko = 0.5)</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>phi Vc &gt;= Vu</t>
+          <t>phi Mn &gt;= Mu (marco cerrado)</t>
         </is>
       </c>
       <c r="D31" s="22">
-        <f>ESTRUCTURAL!B64</f>
+        <f>ESTRUCTURAL!B61</f>
         <v/>
       </c>
       <c r="E31" s="3">
-        <f>IF(ESTRUCTURAL!B64&gt;=ESTRUCTURAL!B63,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B61&gt;=ESTRUCTURAL!B57,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Muro tramo normal: refuerzo en una capa</t>
+          <t>Muro tramo normal: cortante</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 14.3.4 (dos capas solo si e &gt; 0.20 m)</t>
+          <t>RNE E.060 art. 11.3</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>e = 0.15 m: una capa en el eje</t>
+          <t>phi Vc &gt;= Vu</t>
         </is>
       </c>
       <c r="D32" s="22">
-        <f>DATOS!$B$18</f>
+        <f>ESTRUCTURAL!B64</f>
         <v/>
       </c>
       <c r="E32" s="3">
-        <f>IF(DATOS!$B$18&lt;=0.20,"CUMPLE","VERIFICAR")</f>
+        <f>IF(ESTRUCTURAL!B64&gt;=ESTRUCTURAL!B63,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Muro cruce de motos: flexion</t>
+          <t>Muro tramo normal: refuerzo en una capa</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060</t>
+          <t>RNE E.060 art. 14.3.4 (dos capas solo si e &gt; 0.20 m)</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>phi Mn &gt;= Mu</t>
+          <t>e = 0.15 m: una capa en el eje</t>
         </is>
       </c>
       <c r="D33" s="22">
-        <f>ESTRUCTURAL!B72</f>
+        <f>DATOS!$B$18</f>
         <v/>
       </c>
       <c r="E33" s="3">
-        <f>IF(ESTRUCTURAL!B72&gt;=ESTRUCTURAL!B69,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(DATOS!$B$18&lt;=0.20,"CUMPLE","VERIFICAR")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Muro cruce de camiones: flexion (sobrecarga lateral camion)</t>
+          <t>Muro cruce de motos: flexion</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060; AASHTO LRFD 3.11.6.4</t>
+          <t>RNE E.060</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -32032,23 +32082,23 @@
         </is>
       </c>
       <c r="D34" s="22">
-        <f>ESTRUCTURAL!B81</f>
+        <f>ESTRUCTURAL!B72</f>
         <v/>
       </c>
       <c r="E34" s="3">
-        <f>IF(ESTRUCTURAL!B81&gt;=ESTRUCTURAL!B77,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B72&gt;=ESTRUCTURAL!B69,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Losa de fondo: flexion</t>
+          <t>Muro cruce de camiones: flexion (sobrecarga lateral camion)</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060</t>
+          <t>RNE E.060; AASHTO LRFD 3.11.6.4</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -32057,171 +32107,169 @@
         </is>
       </c>
       <c r="D35" s="22">
-        <f>ESTRUCTURAL!B90</f>
+        <f>ESTRUCTURAL!B81</f>
         <v/>
       </c>
       <c r="E35" s="3">
-        <f>IF(ESTRUCTURAL!B90&gt;=ESTRUCTURAL!B86,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B81&gt;=ESTRUCTURAL!B77,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Presion sobre el suelo</t>
+          <t>Losa de fondo: flexion</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>RNE E.050 Suelos y Cimentaciones</t>
+          <t>RNE E.060</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>q &lt;= 0.50 kg/cm2, valor minimo usual de capacidad admisible en suelos blandos; el EMS del proyecto lo confirma</t>
+          <t>phi Mn &gt;= Mu</t>
         </is>
       </c>
       <c r="D36" s="22">
-        <f>ESTRUCTURAL!B91</f>
+        <f>ESTRUCTURAL!B90</f>
         <v/>
       </c>
       <c r="E36" s="3">
-        <f>IF(ESTRUCTURAL!B91&lt;=0.5,"CUMPLE (q = "&amp;TEXT(ESTRUCTURAL!B91,"0.00")&amp;" kg/cm2 &lt; 0.50)","VERIFICAR EMS")</f>
+        <f>IF(ESTRUCTURAL!B90&gt;=ESTRUCTURAL!B86,"CUMPLE","NO CUMPLE")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Tapa de registro 0.68 x 0.68 x 0.08: flexion (rueda liviana)</t>
+          <t>Presion sobre el suelo</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060</t>
+          <t>RNE E.050 Suelos y Cimentaciones</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>phi Mn &gt;= Mu</t>
+          <t>q &lt;= 0.50 kg/cm2, valor minimo usual de capacidad admisible en suelos blandos; el EMS del proyecto lo confirma</t>
         </is>
       </c>
       <c r="D37" s="22">
-        <f>ESTRUCTURAL!B101</f>
+        <f>ESTRUCTURAL!B91</f>
         <v/>
       </c>
       <c r="E37" s="3">
-        <f>IF(ESTRUCTURAL!B101&gt;=ESTRUCTURAL!B97,"CUMPLE","NO CUMPLE")</f>
+        <f>IF(ESTRUCTURAL!B91&lt;=0.5,"CUMPLE (q = "&amp;TEXT(ESTRUCTURAL!B91,"0.00")&amp;" kg/cm2 &lt; 0.50)","VERIFICAR EMS")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Recubrimientos</t>
+          <t>Tapa de registro 0.68 x 0.68 x 0.08: flexion (rueda liviana)</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>RNE E.060 art. 7.7 (concreto sobre solado: 4 cm)</t>
+          <t>RNE E.060</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>4 cm muros y losa de fondo; 2.5 cm losa superior no expuesta; 4 cm cruce de camiones</t>
-        </is>
-      </c>
-      <c r="D38" s="22" t="inlineStr">
-        <is>
-          <t>aplicado</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>CUMPLE</t>
-        </is>
+          <t>phi Mn &gt;= Mu</t>
+        </is>
+      </c>
+      <c r="D38" s="22">
+        <f>ESTRUCTURAL!B101</f>
+        <v/>
+      </c>
+      <c r="E38" s="3">
+        <f>IF(ESTRUCTURAL!B101&gt;=ESTRUCTURAL!B97,"CUMPLE","NO CUMPLE")</f>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
+          <t>Recubrimientos</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>RNE E.060 art. 7.7 (concreto sobre solado: 4 cm)</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>4 cm muros y losa de fondo; 2.5 cm losa superior no expuesta; 4 cm cruce de camiones</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>aplicado</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
           <t>Traslapes y ganchos</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>RNE E.060 cap. 12</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>Traslape 0.40 m (3/8"), 0.50 m (1/2"); ganchos 0.30 m</t>
         </is>
       </c>
-      <c r="D39" s="22" t="inlineStr">
+      <c r="D40" s="22" t="inlineStr">
         <is>
           <t>aplicado</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>CUMPLE</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="12" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>CONSTRUCTIVOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Registros de limpieza</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>RNE CE.040 (accesibilidad para mantenimiento)</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>Separacion &lt;= 12 m y en cada llegada de cuneta; fuera de los cruces vehiculares</t>
-        </is>
-      </c>
-      <c r="D41" s="22" t="inlineStr">
-        <is>
-          <t>7 + 3 registros</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>CUMPLE</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Juntas de dilatacion</t>
+          <t>Registros de limpieza</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Practica del colector receptor (CAR Mujeres)</t>
+          <t>RNE CE.040 (accesibilidad para mantenimiento)</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Cada 4.00 m con tecnopor 1" y sello</t>
+          <t>Separacion &lt;= 12 m y en cada llegada de cuneta; fuera de los cruces vehiculares</t>
         </is>
       </c>
       <c r="D42" s="22" t="inlineStr">
         <is>
-          <t>17 juntas</t>
+          <t>7 + 3 registros</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -32233,80 +32281,107 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
+          <t>Juntas de dilatacion</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Practica del colector receptor (CAR Mujeres)</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Cada 4.00 m con tecnopor 1" y sello</t>
+        </is>
+      </c>
+      <c r="D43" s="22" t="inlineStr">
+        <is>
+          <t>17 juntas</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
           <t>Emplazamiento</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>Lindero y faja de la carretera Oasis</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>Dentro del predio, pegado por fuera del cerco, sin invadir la via</t>
         </is>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D44" s="22" t="inlineStr">
         <is>
           <t>eje a 0.575 m del cerco</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>CUMPLE</t>
         </is>
       </c>
     </row>
-    <row r="44"/>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Requisitos que no cumplen o por verificar</t>
         </is>
       </c>
-      <c r="B45" s="3">
-        <f>COUNTIF(E5:E43,"NO CUMPLE*")+COUNTIF(E5:E43,"VERIFICAR*")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46"/>
-    <row r="47">
-      <c r="A47" s="12" t="inlineStr">
+      <c r="B46" s="3">
+        <f>COUNTIF(E5:E44,"NO CUMPLE*")+COUNTIF(E5:E44,"VERIFICAR*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
         <is>
           <t>DATOS DE OTROS EXPEDIENTES Y COMO QUEDAN CUBIERTOS EN ESTE DISENO</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>1. Cota de llegada del colector del CAR Varones (CUI 2705619): se adopta 260.18 msnm (dato de ese expediente). La caja CL admite cualquier cota entre el nivel de agua en 0+000 + 0.10 y la cara inferior de la losa (ver fila del cuadro); dentro de ese rango no cambia la seccion, el armado ni el metrado.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>2. Caudal del CAR Varones (258.7 L/s): dato de su memoria y base del colector receptor (560.7 L/s). La seccion de este tramo tiene capacidad para mas del doble del caudal de diseno con llenado del 85 % (ver fila del cuadro), de modo que una variacion de ese dato no compromete el tramo.</t>
+          <t>1. Llegada del colector del CAR Varones (CUI 2705619): cota de fondo 259.884 msnm en la cara este de la CL (ventana 0.60 x 1.17 hasta el techo de la CL) y cuneta Eje 01 de Varones por el muro norte (ventana 0.40 x 0.66, NCF 260.394). Como la CL queda del lado de Varones, su tapa se fija en +261.15 (piso de ese proyecto); el colector de Varones entrega 221.7 + 37.0 = 258.7 L/s.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>3. Capacidad portante: la presion transmitida (0.33 kg/cm2) es menor que 0.50 kg/cm2, valor minimo usual de suelos blandos; el EMS del proyecto, exigido por la norma E.050, la confirma.</t>
+          <t>2. Caudal del CAR Varones (258.7 L/s): dato de su memoria y base del colector receptor (560.7 L/s). La seccion de este tramo tiene capacidad para mas del doble del caudal de diseno con llenado del 85 % (ver fila del cuadro), de modo que una variacion de ese dato no compromete el tramo.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>4. Coordenadas UTM: obtenidas del registro R-01 del CAR Mujeres (CUI 2717013) y del rumbo del lindero (azimut 49.54); el trazo queda definido por su posicion fisica (eje a 0.575 m del cerco) y se replantea en obra desde ese cerco.</t>
+          <t>3. Capacidad portante: la presion transmitida (0.33 kg/cm2) es menor que 0.50 kg/cm2, valor minimo usual de suelos blandos; el EMS del proyecto, exigido por la norma E.050, la confirma.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>4. Coordenadas UTM: obtenidas del registro R-01 del CAR Mujeres (CUI 2717013) y del rumbo del lindero (azimut 49.54); el trazo queda definido por su posicion fisica (eje a 0.575 m del cerco) y se replantea en obra desde ese cerco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>5. Cotas de fondo de las cunetas: tomadas del plano de arquitectura vigente (PLANTA GENERAL REFUGIO, 03-10-2026), perfiles 01 a 12; todas caen libremente al colector.</t>
         </is>

</xml_diff>